<commit_message>
add UI use sample
</commit_message>
<xml_diff>
--- a/Templates~/Config/Excels/Test.xlsx
+++ b/Templates~/Config/Excels/Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\Unity\Project Abyss\Config\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\Unity\Game Dev Tools\Client\Packages\com.moirai.framework\Templates~\Config\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB29B059-055A-414B-956A-5ABBA1FB5676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E4C820-D2C9-4BC1-9708-8DD364D6A7EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4980" yWindow="4980" windowWidth="28800" windowHeight="14820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4980" yWindow="4980" windowWidth="28815" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>##type</t>
   </si>
@@ -142,22 +142,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>stats_name_health</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>stats_desc_health</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>stats_name_health1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>stats_desc_health1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>price</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -200,48 +184,23 @@
     <t>25阿达</t>
   </si>
   <si>
-    <t>阿斯顿4</t>
-  </si>
-  <si>
-    <t>26阿达</t>
-  </si>
-  <si>
-    <t>阿斯顿5</t>
-  </si>
-  <si>
-    <t>27阿达</t>
-  </si>
-  <si>
-    <t>28阿达</t>
-  </si>
-  <si>
-    <t>阿斯顿7</t>
-  </si>
-  <si>
-    <t>29阿达</t>
-  </si>
-  <si>
-    <t>阿斯顿8</t>
-  </si>
-  <si>
-    <t>30阿达</t>
-  </si>
-  <si>
-    <t>阿斯顿9</t>
-  </si>
-  <si>
-    <t>31阿达</t>
-  </si>
-  <si>
-    <t>阿斯顿6</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>list,string</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>测试数据</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>test</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_only_zh</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>test_only_en</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -697,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.125" bestFit="1" customWidth="1"/>
@@ -706,7 +665,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -718,10 +677,10 @@
         <v>7</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>15</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>19</v>
       </c>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
@@ -743,7 +702,7 @@
         <v>4</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
@@ -760,7 +719,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="10"/>
@@ -768,7 +727,7 @@
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
@@ -780,10 +739,10 @@
         <v>9</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
@@ -793,10 +752,10 @@
         <v>1001</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -805,21 +764,21 @@
         <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>1002</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E6">
         <v>101</v>
@@ -828,7 +787,7 @@
         <v>124</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -836,10 +795,10 @@
         <v>1003</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E7">
         <v>102</v>
@@ -848,10 +807,10 @@
         <v>125</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -859,10 +818,10 @@
         <v>1004</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E8">
         <v>103</v>
@@ -871,151 +830,10 @@
         <v>126</v>
       </c>
       <c r="G8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B9">
-        <v>1005</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9">
-        <v>104</v>
-      </c>
-      <c r="F9">
-        <v>127</v>
-      </c>
-      <c r="G9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10">
-        <v>1006</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10">
-        <v>105</v>
-      </c>
-      <c r="F10">
-        <v>128</v>
-      </c>
-      <c r="G10" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B11">
-        <v>1007</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11">
-        <v>106</v>
-      </c>
-      <c r="F11">
-        <v>129</v>
-      </c>
-      <c r="G11" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B12">
-        <v>1008</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12">
-        <v>107</v>
-      </c>
-      <c r="F12">
-        <v>130</v>
-      </c>
-      <c r="G12" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B13">
-        <v>1009</v>
-      </c>
-      <c r="C13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13">
-        <v>108</v>
-      </c>
-      <c r="F13">
-        <v>131</v>
-      </c>
-      <c r="G13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B14">
-        <v>1010</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14">
-        <v>109</v>
-      </c>
-      <c r="F14">
-        <v>132</v>
-      </c>
-      <c r="G14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>